<commit_message>
added caspar tsv and md for database
</commit_message>
<xml_diff>
--- a/__READ ME.xlsx
+++ b/__READ ME.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo M1 Trait Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFC0166D-8105-C94E-9079-F4303A09D233}"/>
+  <xr:revisionPtr revIDLastSave="183" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4408D88-2ABD-CF41-9BEE-E64B2B911C6C}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="-21100" windowWidth="27500" windowHeight="19660" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20380" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="206">
   <si>
     <t>Publication CodeName</t>
   </si>
@@ -649,6 +649,12 @@
   </si>
   <si>
     <t>10.3389/fncir.2013.00030</t>
+  </si>
+  <si>
+    <t>save as tsv with DOI plus item for file name</t>
+  </si>
+  <si>
+    <t>--&gt; Online database</t>
   </si>
 </sst>
 </file>
@@ -729,9 +735,11 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1763,7 +1771,7 @@
       <c r="F17" t="s">
         <v>69</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" s="8" t="s">
         <v>170</v>
       </c>
       <c r="H17" s="5"/>
@@ -1799,7 +1807,7 @@
       <c r="F18" t="s">
         <v>69</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" s="8" t="s">
         <v>171</v>
       </c>
       <c r="H18" s="5"/>
@@ -2498,6 +2506,14 @@
       </c>
       <c r="B53" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A54" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B54" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
@@ -2553,6 +2569,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="acb3cbe4b9dee1876b3bbe7116f679b3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ca927c27970307cd175704f09b582c5c" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
@@ -2789,27 +2825,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F6D714A-5497-420A-9146-5640EA73F0F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2826,29 +2867,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added Dos Santos 2020
</commit_message>
<xml_diff>
--- a/__READ ME.xlsx
+++ b/__READ ME.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo M1 Trait Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="227" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0050A280-8D89-8942-BF38-BC48EAE125AF}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67144838-569A-A743-8DAD-DB58B14466F4}"/>
   <bookViews>
-    <workbookView xWindow="42300" yWindow="-5960" windowWidth="38960" windowHeight="20480" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
+    <workbookView xWindow="34960" yWindow="-5960" windowWidth="50800" windowHeight="17920" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="220">
   <si>
     <t>Publication CodeName</t>
   </si>
@@ -209,9 +209,6 @@
     <t>dossantos_etal_2017_primary_or_equivalent.csv</t>
   </si>
   <si>
-    <t>dossantos_etal_2017.csv</t>
-  </si>
-  <si>
     <t>doc, erratum (on pdf)</t>
   </si>
   <si>
@@ -423,9 +420,6 @@
   </si>
   <si>
     <t>number of cortical areas</t>
-  </si>
-  <si>
-    <t>cortical surface area and number of areas (broadly defined)</t>
   </si>
   <si>
     <t>maybe delete: not relevent in current dataset, unless for imputations?</t>
@@ -691,6 +685,18 @@
   </si>
   <si>
     <t>HerculanoHouzel_etal_2015_Table5.csv</t>
+  </si>
+  <si>
+    <t>cerebral cortex surface area and number of areas (broadly defined)</t>
+  </si>
+  <si>
+    <t>dossantos_etal_2020_Table1_primary_or_equivalent.csv</t>
+  </si>
+  <si>
+    <t>dossantos_etal_2020_table1.csv</t>
+  </si>
+  <si>
+    <t>dossantos_etal_2017_tables1.csv</t>
   </si>
 </sst>
 </file>
@@ -1111,14 +1117,14 @@
     <col min="5" max="5" width="23.1640625" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="19.1640625" customWidth="1"/>
-    <col min="8" max="8" width="30.33203125" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
     <col min="9" max="9" width="5.33203125" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
     <col min="11" max="11" width="13.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.6640625" customWidth="1"/>
     <col min="13" max="14" width="22.1640625" customWidth="1"/>
     <col min="15" max="15" width="12.33203125" customWidth="1"/>
-    <col min="18" max="18" width="46.5" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -1126,16 +1132,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -1150,7 +1156,7 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>5</v>
@@ -1215,14 +1221,14 @@
         <v>21</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>140</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>142</v>
       </c>
       <c r="F3" t="s">
         <v>22</v>
@@ -1265,15 +1271,15 @@
         <v>31</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G4" t="s">
         <v>32</v>
@@ -1317,15 +1323,15 @@
         <v>31</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G5" t="s">
         <v>43</v>
@@ -1364,21 +1370,21 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I6" t="s">
         <v>34</v>
@@ -1391,20 +1397,20 @@
         <v>36</v>
       </c>
       <c r="L6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="M6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="N6" s="6"/>
       <c r="O6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="R6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
@@ -1412,15 +1418,15 @@
         <v>49</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" t="s">
@@ -1455,7 +1461,7 @@
         <v>53</v>
       </c>
       <c r="R7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="S7" t="s">
         <v>54</v>
@@ -1466,19 +1472,18 @@
         <v>55</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F8" t="s">
-        <v>200</v>
-      </c>
-      <c r="G8" s="3"/>
+        <v>198</v>
+      </c>
       <c r="H8" t="s">
         <v>56</v>
       </c>
@@ -1486,50 +1491,54 @@
         <v>34</v>
       </c>
       <c r="J8" t="s">
+        <v>219</v>
+      </c>
+      <c r="K8" t="s">
         <v>57</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>58</v>
-      </c>
-      <c r="L8" t="s">
-        <v>59</v>
       </c>
       <c r="M8" t="s">
         <v>46</v>
       </c>
       <c r="N8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="O8" t="s">
         <v>60</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>61</v>
       </c>
-      <c r="P8" t="s">
+      <c r="S8" t="s">
         <v>62</v>
-      </c>
-      <c r="S8" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E9" s="7"/>
-      <c r="F9" s="2" t="s">
-        <v>65</v>
+      <c r="F9" t="s">
+        <v>198</v>
       </c>
       <c r="G9" s="3"/>
-      <c r="H9" s="5"/>
-      <c r="J9">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="H9" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" t="s">
+        <v>218</v>
       </c>
       <c r="K9" t="s">
         <v>36</v>
@@ -1538,33 +1547,33 @@
         <v>26</v>
       </c>
       <c r="O9" t="s">
+        <v>60</v>
+      </c>
+      <c r="P9" t="s">
         <v>61</v>
       </c>
-      <c r="P9" t="s">
-        <v>62</v>
-      </c>
       <c r="S9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E10" s="7"/>
       <c r="F10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I10" t="s">
         <v>34</v>
@@ -1574,7 +1583,7 @@
         <v>Y</v>
       </c>
       <c r="K10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L10" t="s">
         <v>26</v>
@@ -1583,13 +1592,13 @@
         <v>37</v>
       </c>
       <c r="N10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="O10" t="s">
+        <v>216</v>
+      </c>
+      <c r="R10" t="s">
         <v>70</v>
-      </c>
-      <c r="O10" t="s">
-        <v>129</v>
-      </c>
-      <c r="R10" t="s">
-        <v>71</v>
       </c>
       <c r="S10" t="s">
         <v>20</v>
@@ -1597,28 +1606,28 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E11" s="11"/>
       <c r="F11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="I11" t="s">
         <v>34</v>
       </c>
       <c r="J11" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K11" t="s">
         <v>36</v>
@@ -1627,16 +1636,16 @@
         <v>26</v>
       </c>
       <c r="M11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="O11" t="s">
+        <v>73</v>
+      </c>
+      <c r="P11" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q11" t="s">
         <v>74</v>
-      </c>
-      <c r="P11" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>75</v>
       </c>
       <c r="S11" t="s">
         <v>20</v>
@@ -1644,18 +1653,18 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="5"/>
@@ -1670,7 +1679,7 @@
         <v>26</v>
       </c>
       <c r="O12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S12" t="s">
         <v>20</v>
@@ -1678,18 +1687,18 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="5"/>
@@ -1704,7 +1713,7 @@
         <v>26</v>
       </c>
       <c r="O13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S13" t="s">
         <v>42</v>
@@ -1712,30 +1721,30 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>34</v>
       </c>
       <c r="J14" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K14" t="s">
         <v>36</v>
@@ -1747,38 +1756,38 @@
         <v>37</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="J15" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K15" t="s">
         <v>36</v>
@@ -1790,38 +1799,38 @@
         <v>37</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="J16" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="K16" t="s">
         <v>36</v>
@@ -1833,38 +1842,38 @@
         <v>37</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J17" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K17" t="s">
         <v>36</v>
@@ -1876,38 +1885,38 @@
         <v>37</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E18" s="7"/>
       <c r="F18" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="J18" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="K18" t="s">
         <v>36</v>
@@ -1919,32 +1928,32 @@
         <v>37</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="H19" s="5"/>
       <c r="J19">
@@ -1957,30 +1966,33 @@
       <c r="L19" t="s">
         <v>26</v>
       </c>
+      <c r="M19" t="s">
+        <v>130</v>
+      </c>
       <c r="O19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="S19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H20" s="5"/>
       <c r="J20">
@@ -1994,29 +2006,29 @@
         <v>26</v>
       </c>
       <c r="O20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E21" s="7"/>
       <c r="F21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H21" s="5"/>
       <c r="J21">
@@ -2030,29 +2042,29 @@
         <v>26</v>
       </c>
       <c r="O21" t="s">
+        <v>85</v>
+      </c>
+      <c r="S21" t="s">
         <v>86</v>
-      </c>
-      <c r="S21" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H22" s="5"/>
       <c r="J22">
@@ -2066,29 +2078,29 @@
         <v>26</v>
       </c>
       <c r="O22" t="s">
+        <v>85</v>
+      </c>
+      <c r="S22" t="s">
         <v>86</v>
-      </c>
-      <c r="S22" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E23" s="7"/>
       <c r="F23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H23" s="5"/>
       <c r="J23">
@@ -2102,29 +2114,29 @@
         <v>26</v>
       </c>
       <c r="O23" t="s">
+        <v>85</v>
+      </c>
+      <c r="S23" t="s">
         <v>86</v>
-      </c>
-      <c r="S23" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H24" s="5"/>
       <c r="J24">
@@ -2138,26 +2150,26 @@
         <v>26</v>
       </c>
       <c r="O24" t="s">
+        <v>85</v>
+      </c>
+      <c r="S24" t="s">
         <v>86</v>
-      </c>
-      <c r="S24" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="5"/>
@@ -2172,29 +2184,29 @@
         <v>26</v>
       </c>
       <c r="O25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H26" s="5"/>
       <c r="J26">
@@ -2208,29 +2220,29 @@
         <v>26</v>
       </c>
       <c r="O26" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="S26" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H27" s="5"/>
       <c r="J27">
@@ -2244,26 +2256,26 @@
         <v>26</v>
       </c>
       <c r="O27" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="S27" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="5"/>
@@ -2281,16 +2293,16 @@
         <v>46</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="O28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P28" t="s">
         <v>29</v>
       </c>
       <c r="Q28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="S28" t="s">
         <v>42</v>
@@ -2298,20 +2310,20 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="5"/>
@@ -2329,10 +2341,10 @@
         <v>46</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O29" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P29" t="s">
         <v>29</v>
@@ -2346,21 +2358,21 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E30" s="7"/>
       <c r="F30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H30" s="5"/>
       <c r="J30">
@@ -2371,13 +2383,13 @@
         <v>36</v>
       </c>
       <c r="L30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S30" t="s">
         <v>42</v>
@@ -2385,21 +2397,21 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E31" s="7"/>
       <c r="F31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H31" s="5"/>
       <c r="J31">
@@ -2410,13 +2422,13 @@
         <v>36</v>
       </c>
       <c r="L31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="S31" t="s">
         <v>42</v>
@@ -2424,18 +2436,18 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="5"/>
@@ -2447,10 +2459,10 @@
         <v>36</v>
       </c>
       <c r="L32" t="s">
+        <v>99</v>
+      </c>
+      <c r="O32" t="s">
         <v>100</v>
-      </c>
-      <c r="O32" t="s">
-        <v>101</v>
       </c>
       <c r="S32" t="s">
         <v>20</v>
@@ -2458,18 +2470,18 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="5"/>
@@ -2478,13 +2490,13 @@
         <v>0</v>
       </c>
       <c r="K33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L33" t="s">
         <v>26</v>
       </c>
       <c r="O33" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="S33" t="s">
         <v>42</v>
@@ -2492,97 +2504,97 @@
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B44" t="s">
         <v>106</v>
-      </c>
-      <c r="B44" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B45" t="s">
         <v>108</v>
-      </c>
-      <c r="B45" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B46" t="s">
         <v>110</v>
-      </c>
-      <c r="B46" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B47" t="s">
         <v>112</v>
-      </c>
-      <c r="B47" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B48" t="s">
         <v>114</v>
-      </c>
-      <c r="B48" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B49" t="s">
         <v>116</v>
-      </c>
-      <c r="B49" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B50" t="s">
         <v>118</v>
-      </c>
-      <c r="B50" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B51" t="s">
         <v>120</v>
-      </c>
-      <c r="B51" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B52" t="s">
         <v>122</v>
-      </c>
-      <c r="B52" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="10" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B53" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2635,26 +2647,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="acb3cbe4b9dee1876b3bbe7116f679b3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ca927c27970307cd175704f09b582c5c" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
@@ -2891,32 +2883,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F6D714A-5497-420A-9146-5640EA73F0F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2933,4 +2920,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>